<commit_message>
Feat: Event impact modelling commit message
</commit_message>
<xml_diff>
--- a/data/raw/ethiopia_fi_unified_data.xlsx
+++ b/data/raw/ethiopia_fi_unified_data.xlsx
@@ -1,13 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbe\Desktop\week 11\ethiopia_fi_forecast\data\raw\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="5000" activeTab="1"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="ethiopia_fi_unified_data" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Impact_sheet" sheetId="2" r:id="rId6"/>
+    <sheet name="ethiopia_fi_unified_data" sheetId="1" r:id="rId1"/>
+    <sheet name="Impact_sheet" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ethiopia_fi_unified_data!$A$1:$AH$44</definedName>
+  </definedNames>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -965,25 +976,28 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -991,42 +1005,41 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1034,7 +1047,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1224,21 +1237,54 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:AH44"/>
+  <sheetFormatPr defaultColWidth="12.7265625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="5" max="5" width="32.13"/>
-    <col customWidth="1" min="6" max="6" width="20.38"/>
+    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.90625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.6328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="44.36328125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="39.36328125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="36.36328125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="7.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1342,7 +1388,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>34</v>
       </c>
@@ -1362,7 +1408,7 @@
         <v>39</v>
       </c>
       <c r="H2" s="1">
-        <v>22.0</v>
+        <v>22</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>40</v>
@@ -1371,10 +1417,10 @@
         <v>41</v>
       </c>
       <c r="L2" s="2">
-        <v>42004.0</v>
+        <v>42004</v>
       </c>
       <c r="O2" s="1">
-        <v>2014.0</v>
+        <v>2014</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>42</v>
@@ -1398,13 +1444,13 @@
         <v>48</v>
       </c>
       <c r="AE2" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG2" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>50</v>
       </c>
@@ -1424,7 +1470,7 @@
         <v>39</v>
       </c>
       <c r="H3" s="1">
-        <v>35.0</v>
+        <v>35</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>40</v>
@@ -1433,10 +1479,10 @@
         <v>41</v>
       </c>
       <c r="L3" s="2">
-        <v>43100.0</v>
+        <v>43100</v>
       </c>
       <c r="O3" s="1">
-        <v>2017.0</v>
+        <v>2017</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>42</v>
@@ -1460,10 +1506,10 @@
         <v>48</v>
       </c>
       <c r="AE3" s="2">
-        <v>45677.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>45677</v>
+      </c>
+    </row>
+    <row r="4" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>52</v>
       </c>
@@ -1483,7 +1529,7 @@
         <v>39</v>
       </c>
       <c r="H4" s="1">
-        <v>46.0</v>
+        <v>46</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>40</v>
@@ -1492,10 +1538,10 @@
         <v>41</v>
       </c>
       <c r="L4" s="2">
-        <v>44561.0</v>
+        <v>44561</v>
       </c>
       <c r="O4" s="1">
-        <v>2021.0</v>
+        <v>2021</v>
       </c>
       <c r="P4" s="1" t="s">
         <v>42</v>
@@ -1519,10 +1565,10 @@
         <v>48</v>
       </c>
       <c r="AE4" s="2">
-        <v>45677.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>45677</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>54</v>
       </c>
@@ -1542,7 +1588,7 @@
         <v>39</v>
       </c>
       <c r="H5" s="1">
-        <v>56.0</v>
+        <v>56</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>40</v>
@@ -1551,10 +1597,10 @@
         <v>41</v>
       </c>
       <c r="L5" s="2">
-        <v>44561.0</v>
+        <v>44561</v>
       </c>
       <c r="O5" s="1">
-        <v>2021.0</v>
+        <v>2021</v>
       </c>
       <c r="P5" s="1" t="s">
         <v>55</v>
@@ -1578,13 +1624,13 @@
         <v>48</v>
       </c>
       <c r="AE5" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG5" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>57</v>
       </c>
@@ -1604,7 +1650,7 @@
         <v>39</v>
       </c>
       <c r="H6" s="1">
-        <v>36.0</v>
+        <v>36</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>40</v>
@@ -1613,10 +1659,10 @@
         <v>41</v>
       </c>
       <c r="L6" s="2">
-        <v>44561.0</v>
+        <v>44561</v>
       </c>
       <c r="O6" s="1">
-        <v>2021.0</v>
+        <v>2021</v>
       </c>
       <c r="P6" s="1" t="s">
         <v>58</v>
@@ -1640,13 +1686,13 @@
         <v>48</v>
       </c>
       <c r="AE6" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG6" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>59</v>
       </c>
@@ -1666,7 +1712,7 @@
         <v>39</v>
       </c>
       <c r="H7" s="1">
-        <v>49.0</v>
+        <v>49</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>40</v>
@@ -1675,16 +1721,16 @@
         <v>41</v>
       </c>
       <c r="L7" s="2">
-        <v>45625.0</v>
+        <v>45625</v>
       </c>
       <c r="M7" s="2">
-        <v>45580.0</v>
+        <v>45580</v>
       </c>
       <c r="N7" s="2">
-        <v>45625.0</v>
+        <v>45625</v>
       </c>
       <c r="O7" s="1">
-        <v>2024.0</v>
+        <v>2024</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>42</v>
@@ -1708,7 +1754,7 @@
         <v>48</v>
       </c>
       <c r="AE7" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AF7" s="1" t="s">
         <v>61</v>
@@ -1717,7 +1763,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>63</v>
       </c>
@@ -1746,10 +1792,10 @@
         <v>41</v>
       </c>
       <c r="L8" s="2">
-        <v>44561.0</v>
+        <v>44561</v>
       </c>
       <c r="O8" s="1">
-        <v>2021.0</v>
+        <v>2021</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>42</v>
@@ -1773,10 +1819,10 @@
         <v>48</v>
       </c>
       <c r="AE8" s="2">
-        <v>45677.0</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>45677</v>
+      </c>
+    </row>
+    <row r="9" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>66</v>
       </c>
@@ -1796,7 +1842,7 @@
         <v>39</v>
       </c>
       <c r="H9" s="1">
-        <v>9.45</v>
+        <v>9.4499999999999993</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>40</v>
@@ -1805,10 +1851,10 @@
         <v>41</v>
       </c>
       <c r="L9" s="2">
-        <v>45625.0</v>
+        <v>45625</v>
       </c>
       <c r="O9" s="1">
-        <v>2024.0</v>
+        <v>2024</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>42</v>
@@ -1832,13 +1878,13 @@
         <v>48</v>
       </c>
       <c r="AE9" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG9" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>68</v>
       </c>
@@ -1867,7 +1913,7 @@
         <v>41</v>
       </c>
       <c r="L10" s="2">
-        <v>45107.0</v>
+        <v>45107</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>71</v>
@@ -1894,13 +1940,13 @@
         <v>48</v>
       </c>
       <c r="AE10" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG10" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>76</v>
       </c>
@@ -1929,7 +1975,7 @@
         <v>41</v>
       </c>
       <c r="L11" s="2">
-        <v>45838.0</v>
+        <v>45838</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>77</v>
@@ -1956,7 +2002,7 @@
         <v>48</v>
       </c>
       <c r="AE11" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AF11" s="1" t="s">
         <v>78</v>
@@ -1965,7 +2011,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>80</v>
       </c>
@@ -1994,10 +2040,10 @@
         <v>41</v>
       </c>
       <c r="L12" s="2">
-        <v>46022.0</v>
+        <v>46022</v>
       </c>
       <c r="O12" s="1">
-        <v>2025.0</v>
+        <v>2025</v>
       </c>
       <c r="P12" s="1" t="s">
         <v>42</v>
@@ -2021,13 +2067,13 @@
         <v>48</v>
       </c>
       <c r="AE12" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG12" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>87</v>
       </c>
@@ -2047,7 +2093,7 @@
         <v>39</v>
       </c>
       <c r="H13" s="1">
-        <v>8000000.0</v>
+        <v>8000000</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>90</v>
@@ -2056,10 +2102,10 @@
         <v>91</v>
       </c>
       <c r="L13" s="2">
-        <v>45519.0</v>
+        <v>45519</v>
       </c>
       <c r="O13" s="1">
-        <v>2024.0</v>
+        <v>2024</v>
       </c>
       <c r="P13" s="1" t="s">
         <v>42</v>
@@ -2083,10 +2129,10 @@
         <v>48</v>
       </c>
       <c r="AE13" s="2">
-        <v>45677.0</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>45677</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>95</v>
       </c>
@@ -2106,7 +2152,7 @@
         <v>39</v>
       </c>
       <c r="H14" s="1">
-        <v>1.2E7</v>
+        <v>12000000</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>90</v>
@@ -2115,10 +2161,10 @@
         <v>91</v>
       </c>
       <c r="L14" s="2">
-        <v>45716.0</v>
+        <v>45716</v>
       </c>
       <c r="O14" s="1">
-        <v>2025.0</v>
+        <v>2025</v>
       </c>
       <c r="P14" s="1" t="s">
         <v>42</v>
@@ -2139,13 +2185,13 @@
         <v>48</v>
       </c>
       <c r="AE14" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AF14" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>98</v>
       </c>
@@ -2165,7 +2211,7 @@
         <v>39</v>
       </c>
       <c r="H15" s="1">
-        <v>1.5E7</v>
+        <v>15000000</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>90</v>
@@ -2174,10 +2220,10 @@
         <v>91</v>
       </c>
       <c r="L15" s="2">
-        <v>45792.0</v>
+        <v>45792</v>
       </c>
       <c r="O15" s="1">
-        <v>2025.0</v>
+        <v>2025</v>
       </c>
       <c r="P15" s="1" t="s">
         <v>42</v>
@@ -2201,10 +2247,10 @@
         <v>48</v>
       </c>
       <c r="AE15" s="2">
-        <v>45677.0</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>45677</v>
+      </c>
+    </row>
+    <row r="16" spans="1:34" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>100</v>
       </c>
@@ -2224,7 +2270,7 @@
         <v>39</v>
       </c>
       <c r="H16" s="1">
-        <v>4.97E7</v>
+        <v>49700000</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>90</v>
@@ -2233,13 +2279,13 @@
         <v>104</v>
       </c>
       <c r="L16" s="2">
-        <v>45480.0</v>
+        <v>45480</v>
       </c>
       <c r="M16" s="2">
-        <v>45115.0</v>
+        <v>45115</v>
       </c>
       <c r="N16" s="2">
-        <v>45480.0</v>
+        <v>45480</v>
       </c>
       <c r="O16" s="1" t="s">
         <v>105</v>
@@ -2266,13 +2312,13 @@
         <v>48</v>
       </c>
       <c r="AE16" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG16" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>109</v>
       </c>
@@ -2292,7 +2338,7 @@
         <v>39</v>
       </c>
       <c r="H17" s="1">
-        <v>1.283E8</v>
+        <v>128300000</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>90</v>
@@ -2301,13 +2347,13 @@
         <v>104</v>
       </c>
       <c r="L17" s="2">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="M17" s="2">
-        <v>45481.0</v>
+        <v>45481</v>
       </c>
       <c r="N17" s="2">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="O17" s="1" t="s">
         <v>77</v>
@@ -2334,7 +2380,7 @@
         <v>48</v>
       </c>
       <c r="AE17" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AF17" s="1" t="s">
         <v>110</v>
@@ -2343,7 +2389,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>112</v>
       </c>
@@ -2363,7 +2409,7 @@
         <v>39</v>
       </c>
       <c r="H18" s="1">
-        <v>5.777E11</v>
+        <v>577700000000</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>115</v>
@@ -2372,13 +2418,13 @@
         <v>116</v>
       </c>
       <c r="L18" s="2">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="M18" s="2">
-        <v>45481.0</v>
+        <v>45481</v>
       </c>
       <c r="N18" s="2">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="O18" s="1" t="s">
         <v>77</v>
@@ -2405,7 +2451,7 @@
         <v>48</v>
       </c>
       <c r="AE18" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AF18" s="1" t="s">
         <v>117</v>
@@ -2414,7 +2460,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>119</v>
       </c>
@@ -2434,7 +2480,7 @@
         <v>122</v>
       </c>
       <c r="H19" s="1">
-        <v>1.193E8</v>
+        <v>119300000</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>90</v>
@@ -2443,13 +2489,13 @@
         <v>104</v>
       </c>
       <c r="L19" s="2">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="M19" s="2">
-        <v>45481.0</v>
+        <v>45481</v>
       </c>
       <c r="N19" s="2">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="O19" s="1" t="s">
         <v>77</v>
@@ -2476,13 +2522,13 @@
         <v>48</v>
       </c>
       <c r="AE19" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG19" s="1" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>124</v>
       </c>
@@ -2502,7 +2548,7 @@
         <v>122</v>
       </c>
       <c r="H20" s="1">
-        <v>1.561E11</v>
+        <v>156100000000</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>115</v>
@@ -2511,13 +2557,13 @@
         <v>116</v>
       </c>
       <c r="L20" s="2">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="M20" s="2">
-        <v>45481.0</v>
+        <v>45481</v>
       </c>
       <c r="N20" s="2">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="O20" s="1" t="s">
         <v>77</v>
@@ -2544,10 +2590,10 @@
         <v>48</v>
       </c>
       <c r="AE20" s="2">
-        <v>45677.0</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>45677</v>
+      </c>
+    </row>
+    <row r="21" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>127</v>
       </c>
@@ -2576,13 +2622,13 @@
         <v>130</v>
       </c>
       <c r="L21" s="2">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="M21" s="2">
-        <v>45481.0</v>
+        <v>45481</v>
       </c>
       <c r="N21" s="2">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="O21" s="1" t="s">
         <v>77</v>
@@ -2606,13 +2652,13 @@
         <v>48</v>
       </c>
       <c r="AE21" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG21" s="1" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>134</v>
       </c>
@@ -2632,7 +2678,7 @@
         <v>39</v>
       </c>
       <c r="H22" s="1">
-        <v>5.484E7</v>
+        <v>54840000</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>90</v>
@@ -2641,13 +2687,13 @@
         <v>137</v>
       </c>
       <c r="L22" s="2">
-        <v>45838.0</v>
+        <v>45838</v>
       </c>
       <c r="M22" s="2">
-        <v>45481.0</v>
+        <v>45481</v>
       </c>
       <c r="N22" s="2">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="O22" s="1" t="s">
         <v>77</v>
@@ -2674,13 +2720,13 @@
         <v>48</v>
       </c>
       <c r="AE22" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AF22" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>140</v>
       </c>
@@ -2700,7 +2746,7 @@
         <v>39</v>
       </c>
       <c r="H23" s="1">
-        <v>2.38E12</v>
+        <v>2380000000000</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>115</v>
@@ -2709,13 +2755,13 @@
         <v>116</v>
       </c>
       <c r="L23" s="2">
-        <v>45838.0</v>
+        <v>45838</v>
       </c>
       <c r="M23" s="2">
-        <v>45481.0</v>
+        <v>45481</v>
       </c>
       <c r="N23" s="2">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="O23" s="1" t="s">
         <v>77</v>
@@ -2742,13 +2788,13 @@
         <v>48</v>
       </c>
       <c r="AE23" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AF23" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>144</v>
       </c>
@@ -2768,7 +2814,7 @@
         <v>39</v>
       </c>
       <c r="H24" s="1">
-        <v>1.08E7</v>
+        <v>10800000</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>90</v>
@@ -2777,10 +2823,10 @@
         <v>137</v>
       </c>
       <c r="L24" s="2">
-        <v>45657.0</v>
+        <v>45657</v>
       </c>
       <c r="O24" s="1">
-        <v>2024.0</v>
+        <v>2024</v>
       </c>
       <c r="P24" s="1" t="s">
         <v>42</v>
@@ -2801,13 +2847,13 @@
         <v>48</v>
       </c>
       <c r="AE24" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AF24" s="1" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>149</v>
       </c>
@@ -2827,7 +2873,7 @@
         <v>39</v>
       </c>
       <c r="H25" s="1">
-        <v>7100000.0</v>
+        <v>7100000</v>
       </c>
       <c r="J25" s="1" t="s">
         <v>90</v>
@@ -2836,10 +2882,10 @@
         <v>137</v>
       </c>
       <c r="L25" s="2">
-        <v>45657.0</v>
+        <v>45657</v>
       </c>
       <c r="O25" s="1">
-        <v>2024.0</v>
+        <v>2024</v>
       </c>
       <c r="P25" s="1" t="s">
         <v>42</v>
@@ -2860,7 +2906,7 @@
         <v>48</v>
       </c>
       <c r="AE25" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AF25" s="1" t="s">
         <v>152</v>
@@ -2869,7 +2915,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>154</v>
       </c>
@@ -2889,7 +2935,7 @@
         <v>39</v>
       </c>
       <c r="H26" s="1">
-        <v>66.0</v>
+        <v>66</v>
       </c>
       <c r="J26" s="1" t="s">
         <v>40</v>
@@ -2898,10 +2944,10 @@
         <v>41</v>
       </c>
       <c r="L26" s="2">
-        <v>45657.0</v>
+        <v>45657</v>
       </c>
       <c r="O26" s="1">
-        <v>2024.0</v>
+        <v>2024</v>
       </c>
       <c r="P26" s="1" t="s">
         <v>42</v>
@@ -2922,13 +2968,13 @@
         <v>48</v>
       </c>
       <c r="AE26" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG26" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>158</v>
       </c>
@@ -2948,7 +2994,7 @@
         <v>162</v>
       </c>
       <c r="H27" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>40</v>
@@ -2957,10 +3003,10 @@
         <v>163</v>
       </c>
       <c r="L27" s="2">
-        <v>45657.0</v>
+        <v>45657</v>
       </c>
       <c r="O27" s="1">
-        <v>2024.0</v>
+        <v>2024</v>
       </c>
       <c r="P27" s="1" t="s">
         <v>42</v>
@@ -2984,13 +3030,13 @@
         <v>48</v>
       </c>
       <c r="AE27" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG27" s="1" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>168</v>
       </c>
@@ -3010,7 +3056,7 @@
         <v>162</v>
       </c>
       <c r="H28" s="1">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="J28" s="1" t="s">
         <v>172</v>
@@ -3019,10 +3065,10 @@
         <v>173</v>
       </c>
       <c r="L28" s="2">
-        <v>44561.0</v>
+        <v>44561</v>
       </c>
       <c r="O28" s="1">
-        <v>2021.0</v>
+        <v>2021</v>
       </c>
       <c r="P28" s="1" t="s">
         <v>42</v>
@@ -3046,13 +3092,13 @@
         <v>48</v>
       </c>
       <c r="AE28" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG28" s="1" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>175</v>
       </c>
@@ -3072,7 +3118,7 @@
         <v>162</v>
       </c>
       <c r="H29" s="1">
-        <v>18.0</v>
+        <v>18</v>
       </c>
       <c r="J29" s="1" t="s">
         <v>172</v>
@@ -3081,10 +3127,10 @@
         <v>173</v>
       </c>
       <c r="L29" s="2">
-        <v>45625.0</v>
+        <v>45625</v>
       </c>
       <c r="O29" s="1">
-        <v>2024.0</v>
+        <v>2024</v>
       </c>
       <c r="P29" s="1" t="s">
         <v>42</v>
@@ -3108,13 +3154,13 @@
         <v>48</v>
       </c>
       <c r="AE29" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG29" s="1" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>177</v>
       </c>
@@ -3134,7 +3180,7 @@
         <v>39</v>
       </c>
       <c r="H30" s="1">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="J30" s="1" t="s">
         <v>40</v>
@@ -3143,10 +3189,10 @@
         <v>41</v>
       </c>
       <c r="L30" s="2">
-        <v>45657.0</v>
+        <v>45657</v>
       </c>
       <c r="O30" s="1">
-        <v>2024.0</v>
+        <v>2024</v>
       </c>
       <c r="P30" s="1" t="s">
         <v>58</v>
@@ -3170,7 +3216,7 @@
         <v>48</v>
       </c>
       <c r="AE30" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AF30" s="1" t="s">
         <v>182</v>
@@ -3179,7 +3225,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>184</v>
       </c>
@@ -3199,7 +3245,7 @@
         <v>162</v>
       </c>
       <c r="H31" s="1">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="J31" s="1" t="s">
         <v>40</v>
@@ -3208,10 +3254,10 @@
         <v>41</v>
       </c>
       <c r="L31" s="2">
-        <v>45657.0</v>
+        <v>45657</v>
       </c>
       <c r="O31" s="1">
-        <v>2024.0</v>
+        <v>2024</v>
       </c>
       <c r="P31" s="1" t="s">
         <v>42</v>
@@ -3235,13 +3281,13 @@
         <v>48</v>
       </c>
       <c r="AE31" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG31" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>190</v>
       </c>
@@ -3261,7 +3307,7 @@
         <v>39</v>
       </c>
       <c r="H32" s="1">
-        <v>70.0</v>
+        <v>70</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>40</v>
@@ -3270,10 +3316,10 @@
         <v>41</v>
       </c>
       <c r="L32" s="2">
-        <v>46022.0</v>
+        <v>46022</v>
       </c>
       <c r="O32" s="1">
-        <v>2025.0</v>
+        <v>2025</v>
       </c>
       <c r="P32" s="1" t="s">
         <v>42</v>
@@ -3297,13 +3343,13 @@
         <v>48</v>
       </c>
       <c r="AE32" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG32" s="1" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>195</v>
       </c>
@@ -3323,7 +3369,7 @@
         <v>39</v>
       </c>
       <c r="H33" s="1">
-        <v>9.0E7</v>
+        <v>90000000</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>90</v>
@@ -3332,10 +3378,10 @@
         <v>91</v>
       </c>
       <c r="L33" s="2">
-        <v>47118.0</v>
+        <v>47118</v>
       </c>
       <c r="O33" s="1">
-        <v>2028.0</v>
+        <v>2028</v>
       </c>
       <c r="P33" s="1" t="s">
         <v>42</v>
@@ -3359,13 +3405,13 @@
         <v>48</v>
       </c>
       <c r="AE33" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG33" s="1" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>198</v>
       </c>
@@ -3385,7 +3431,7 @@
         <v>39</v>
       </c>
       <c r="H34" s="1">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>40</v>
@@ -3394,10 +3440,10 @@
         <v>41</v>
       </c>
       <c r="L34" s="2">
-        <v>47848.0</v>
+        <v>47848</v>
       </c>
       <c r="O34" s="1">
-        <v>2030.0</v>
+        <v>2030</v>
       </c>
       <c r="P34" s="1" t="s">
         <v>58</v>
@@ -3418,13 +3464,13 @@
         <v>48</v>
       </c>
       <c r="AE34" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG34" s="1" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>201</v>
       </c>
@@ -3447,10 +3493,10 @@
         <v>207</v>
       </c>
       <c r="L35" s="2">
-        <v>44333.0</v>
+        <v>44333</v>
       </c>
       <c r="O35" s="1">
-        <v>2021.0</v>
+        <v>2021</v>
       </c>
       <c r="P35" s="1" t="s">
         <v>42</v>
@@ -3474,13 +3520,13 @@
         <v>48</v>
       </c>
       <c r="AE35" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG35" s="1" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>210</v>
       </c>
@@ -3503,10 +3549,10 @@
         <v>207</v>
       </c>
       <c r="L36" s="2">
-        <v>44774.0</v>
+        <v>44774</v>
       </c>
       <c r="O36" s="1">
-        <v>2022.0</v>
+        <v>2022</v>
       </c>
       <c r="P36" s="1" t="s">
         <v>42</v>
@@ -3527,13 +3573,13 @@
         <v>48</v>
       </c>
       <c r="AE36" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG36" s="1" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>217</v>
       </c>
@@ -3556,10 +3602,10 @@
         <v>207</v>
       </c>
       <c r="L37" s="2">
-        <v>45139.0</v>
+        <v>45139</v>
       </c>
       <c r="O37" s="1">
-        <v>2023.0</v>
+        <v>2023</v>
       </c>
       <c r="P37" s="1" t="s">
         <v>42</v>
@@ -3580,13 +3626,13 @@
         <v>48</v>
       </c>
       <c r="AE37" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG37" s="1" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>222</v>
       </c>
@@ -3609,10 +3655,10 @@
         <v>207</v>
       </c>
       <c r="L38" s="2">
-        <v>45292.0</v>
+        <v>45292</v>
       </c>
       <c r="O38" s="1">
-        <v>2024.0</v>
+        <v>2024</v>
       </c>
       <c r="P38" s="1" t="s">
         <v>42</v>
@@ -3636,13 +3682,13 @@
         <v>48</v>
       </c>
       <c r="AE38" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG38" s="1" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>228</v>
       </c>
@@ -3665,10 +3711,10 @@
         <v>207</v>
       </c>
       <c r="L39" s="2">
-        <v>45502.0</v>
+        <v>45502</v>
       </c>
       <c r="O39" s="1">
-        <v>2024.0</v>
+        <v>2024</v>
       </c>
       <c r="P39" s="1" t="s">
         <v>42</v>
@@ -3689,13 +3735,13 @@
         <v>48</v>
       </c>
       <c r="AE39" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG39" s="1" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>233</v>
       </c>
@@ -3718,7 +3764,7 @@
         <v>207</v>
       </c>
       <c r="L40" s="2">
-        <v>45566.0</v>
+        <v>45566</v>
       </c>
       <c r="O40" s="1" t="s">
         <v>77</v>
@@ -3745,13 +3791,13 @@
         <v>48</v>
       </c>
       <c r="AE40" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG40" s="1" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>240</v>
       </c>
@@ -3774,7 +3820,7 @@
         <v>207</v>
       </c>
       <c r="L41" s="2">
-        <v>45957.0</v>
+        <v>45957</v>
       </c>
       <c r="O41" s="1" t="s">
         <v>244</v>
@@ -3798,13 +3844,13 @@
         <v>48</v>
       </c>
       <c r="AE41" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG41" s="1" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>246</v>
       </c>
@@ -3827,7 +3873,7 @@
         <v>207</v>
       </c>
       <c r="L42" s="2">
-        <v>46009.0</v>
+        <v>46009</v>
       </c>
       <c r="O42" s="1" t="s">
         <v>244</v>
@@ -3851,13 +3897,13 @@
         <v>48</v>
       </c>
       <c r="AE42" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG42" s="1" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>251</v>
       </c>
@@ -3880,16 +3926,16 @@
         <v>207</v>
       </c>
       <c r="L43" s="2">
-        <v>44440.0</v>
+        <v>44440</v>
       </c>
       <c r="M43" s="2">
-        <v>44440.0</v>
+        <v>44440</v>
       </c>
       <c r="N43" s="2">
-        <v>45838.0</v>
+        <v>45838</v>
       </c>
       <c r="O43" s="1">
-        <v>2021.0</v>
+        <v>2021</v>
       </c>
       <c r="P43" s="1" t="s">
         <v>42</v>
@@ -3913,13 +3959,13 @@
         <v>48</v>
       </c>
       <c r="AE43" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG43" s="1" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:33" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>255</v>
       </c>
@@ -3942,10 +3988,10 @@
         <v>207</v>
       </c>
       <c r="L44" s="2">
-        <v>46006.0</v>
+        <v>46006</v>
       </c>
       <c r="O44" s="1">
-        <v>2025.0</v>
+        <v>2025</v>
       </c>
       <c r="P44" s="1" t="s">
         <v>42</v>
@@ -3966,58 +4012,97 @@
         <v>48</v>
       </c>
       <c r="AE44" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AG44" s="1" t="s">
         <v>259</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AH44"/>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="U2"/>
-    <hyperlink r:id="rId2" ref="U3"/>
-    <hyperlink r:id="rId3" ref="U4"/>
-    <hyperlink r:id="rId4" ref="U5"/>
-    <hyperlink r:id="rId5" ref="U6"/>
-    <hyperlink r:id="rId6" ref="U7"/>
-    <hyperlink r:id="rId7" ref="U8"/>
-    <hyperlink r:id="rId8" ref="U9"/>
-    <hyperlink r:id="rId9" ref="U10"/>
-    <hyperlink r:id="rId10" ref="U11"/>
-    <hyperlink r:id="rId11" ref="U12"/>
-    <hyperlink r:id="rId12" ref="U13"/>
-    <hyperlink r:id="rId13" ref="U15"/>
-    <hyperlink r:id="rId14" ref="U16"/>
-    <hyperlink r:id="rId15" ref="U17"/>
-    <hyperlink r:id="rId16" ref="U18"/>
-    <hyperlink r:id="rId17" ref="U19"/>
-    <hyperlink r:id="rId18" ref="U20"/>
-    <hyperlink r:id="rId19" ref="U22"/>
-    <hyperlink r:id="rId20" ref="U23"/>
-    <hyperlink r:id="rId21" ref="U27"/>
-    <hyperlink r:id="rId22" ref="U28"/>
-    <hyperlink r:id="rId23" ref="U29"/>
-    <hyperlink r:id="rId24" ref="U30"/>
-    <hyperlink r:id="rId25" ref="U31"/>
-    <hyperlink r:id="rId26" ref="U32"/>
-    <hyperlink r:id="rId27" ref="U33"/>
-    <hyperlink r:id="rId28" ref="U35"/>
-    <hyperlink r:id="rId29" ref="U38"/>
-    <hyperlink r:id="rId30" ref="U40"/>
-    <hyperlink r:id="rId31" ref="U43"/>
+    <hyperlink ref="U2" r:id="rId1"/>
+    <hyperlink ref="U3" r:id="rId2"/>
+    <hyperlink ref="U4" r:id="rId3"/>
+    <hyperlink ref="U5" r:id="rId4"/>
+    <hyperlink ref="U6" r:id="rId5"/>
+    <hyperlink ref="U7" r:id="rId6"/>
+    <hyperlink ref="U8" r:id="rId7"/>
+    <hyperlink ref="U9" r:id="rId8"/>
+    <hyperlink ref="U10" r:id="rId9"/>
+    <hyperlink ref="U11" r:id="rId10"/>
+    <hyperlink ref="U12" r:id="rId11"/>
+    <hyperlink ref="U13" r:id="rId12"/>
+    <hyperlink ref="U15" r:id="rId13"/>
+    <hyperlink ref="U16" r:id="rId14"/>
+    <hyperlink ref="U17" r:id="rId15"/>
+    <hyperlink ref="U18" r:id="rId16"/>
+    <hyperlink ref="U19" r:id="rId17"/>
+    <hyperlink ref="U20" r:id="rId18"/>
+    <hyperlink ref="U22" r:id="rId19"/>
+    <hyperlink ref="U23" r:id="rId20"/>
+    <hyperlink ref="U27" r:id="rId21"/>
+    <hyperlink ref="U28" r:id="rId22"/>
+    <hyperlink ref="U29" r:id="rId23"/>
+    <hyperlink ref="U30" r:id="rId24"/>
+    <hyperlink ref="U31" r:id="rId25"/>
+    <hyperlink ref="U32" r:id="rId26"/>
+    <hyperlink ref="U33" r:id="rId27"/>
+    <hyperlink ref="U35" r:id="rId28"/>
+    <hyperlink ref="U38" r:id="rId29"/>
+    <hyperlink ref="U40" r:id="rId30"/>
+    <hyperlink ref="U43" r:id="rId31"/>
   </hyperlinks>
-  <drawing r:id="rId32"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:AI15"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.90625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.6328125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="42.6328125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4124,7 +4209,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>261</v>
       </c>
@@ -4141,7 +4226,7 @@
         <v>263</v>
       </c>
       <c r="I2" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>40</v>
@@ -4150,7 +4235,7 @@
         <v>41</v>
       </c>
       <c r="M2" s="2">
-        <v>44333.0</v>
+        <v>44333</v>
       </c>
       <c r="Q2" s="1" t="s">
         <v>42</v>
@@ -4174,10 +4259,10 @@
         <v>47</v>
       </c>
       <c r="AB2" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="AC2" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="AD2" s="1" t="s">
         <v>266</v>
@@ -4189,13 +4274,13 @@
         <v>48</v>
       </c>
       <c r="AG2" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI2" s="1" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>269</v>
       </c>
@@ -4218,7 +4303,7 @@
         <v>137</v>
       </c>
       <c r="M3" s="2">
-        <v>44333.0</v>
+        <v>44333</v>
       </c>
       <c r="Q3" s="1" t="s">
         <v>42</v>
@@ -4242,7 +4327,7 @@
         <v>47</v>
       </c>
       <c r="AC3" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="AD3" s="1" t="s">
         <v>271</v>
@@ -4251,13 +4336,13 @@
         <v>48</v>
       </c>
       <c r="AG3" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI3" s="1" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>273</v>
       </c>
@@ -4274,7 +4359,7 @@
         <v>274</v>
       </c>
       <c r="I4" s="1">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>40</v>
@@ -4283,7 +4368,7 @@
         <v>41</v>
       </c>
       <c r="M4" s="2">
-        <v>44333.0</v>
+        <v>44333</v>
       </c>
       <c r="Q4" s="1" t="s">
         <v>42</v>
@@ -4307,10 +4392,10 @@
         <v>47</v>
       </c>
       <c r="AB4" s="1">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="AC4" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>271</v>
@@ -4319,13 +4404,13 @@
         <v>48</v>
       </c>
       <c r="AG4" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI4" s="1" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>276</v>
       </c>
@@ -4342,7 +4427,7 @@
         <v>277</v>
       </c>
       <c r="I5" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>40</v>
@@ -4351,7 +4436,7 @@
         <v>41</v>
       </c>
       <c r="M5" s="2">
-        <v>44774.0</v>
+        <v>44774</v>
       </c>
       <c r="Q5" s="1" t="s">
         <v>42</v>
@@ -4375,10 +4460,10 @@
         <v>166</v>
       </c>
       <c r="AB5" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="AC5" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="AD5" s="1" t="s">
         <v>271</v>
@@ -4387,13 +4472,13 @@
         <v>48</v>
       </c>
       <c r="AG5" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI5" s="1" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>279</v>
       </c>
@@ -4410,7 +4495,7 @@
         <v>280</v>
       </c>
       <c r="I6" s="1">
-        <v>-20.0</v>
+        <v>-20</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>40</v>
@@ -4419,7 +4504,7 @@
         <v>41</v>
       </c>
       <c r="M6" s="2">
-        <v>44774.0</v>
+        <v>44774</v>
       </c>
       <c r="Q6" s="1" t="s">
         <v>42</v>
@@ -4443,10 +4528,10 @@
         <v>166</v>
       </c>
       <c r="AB6" s="1">
-        <v>-20.0</v>
+        <v>-20</v>
       </c>
       <c r="AC6" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="AD6" s="1" t="s">
         <v>266</v>
@@ -4458,13 +4543,13 @@
         <v>48</v>
       </c>
       <c r="AG6" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI6" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>285</v>
       </c>
@@ -4487,7 +4572,7 @@
         <v>137</v>
       </c>
       <c r="M7" s="2">
-        <v>45139.0</v>
+        <v>45139</v>
       </c>
       <c r="Q7" s="1" t="s">
         <v>42</v>
@@ -4511,7 +4596,7 @@
         <v>47</v>
       </c>
       <c r="AC7" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="AD7" s="1" t="s">
         <v>271</v>
@@ -4520,13 +4605,13 @@
         <v>48</v>
       </c>
       <c r="AG7" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI7" s="1" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>287</v>
       </c>
@@ -4543,7 +4628,7 @@
         <v>288</v>
       </c>
       <c r="I8" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>40</v>
@@ -4552,7 +4637,7 @@
         <v>41</v>
       </c>
       <c r="M8" s="2">
-        <v>45139.0</v>
+        <v>45139</v>
       </c>
       <c r="Q8" s="1" t="s">
         <v>42</v>
@@ -4576,10 +4661,10 @@
         <v>166</v>
       </c>
       <c r="AB8" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="AC8" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="AD8" s="1" t="s">
         <v>289</v>
@@ -4588,13 +4673,13 @@
         <v>48</v>
       </c>
       <c r="AG8" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI8" s="1" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>291</v>
       </c>
@@ -4611,7 +4696,7 @@
         <v>292</v>
       </c>
       <c r="I9" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>40</v>
@@ -4620,7 +4705,7 @@
         <v>41</v>
       </c>
       <c r="M9" s="2">
-        <v>45292.0</v>
+        <v>45292</v>
       </c>
       <c r="Q9" s="1" t="s">
         <v>42</v>
@@ -4644,10 +4729,10 @@
         <v>166</v>
       </c>
       <c r="AB9" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="AC9" s="1">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="AD9" s="1" t="s">
         <v>266</v>
@@ -4659,13 +4744,13 @@
         <v>48</v>
       </c>
       <c r="AG9" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>296</v>
       </c>
@@ -4682,7 +4767,7 @@
         <v>297</v>
       </c>
       <c r="I10" s="1">
-        <v>-5.0</v>
+        <v>-5</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>172</v>
@@ -4691,7 +4776,7 @@
         <v>173</v>
       </c>
       <c r="M10" s="2">
-        <v>45292.0</v>
+        <v>45292</v>
       </c>
       <c r="Q10" s="1" t="s">
         <v>42</v>
@@ -4715,10 +4800,10 @@
         <v>166</v>
       </c>
       <c r="AB10" s="1">
-        <v>-5.0</v>
+        <v>-5</v>
       </c>
       <c r="AC10" s="1">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="AD10" s="1" t="s">
         <v>266</v>
@@ -4730,13 +4815,13 @@
         <v>48</v>
       </c>
       <c r="AG10" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI10" s="1" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>299</v>
       </c>
@@ -4753,7 +4838,7 @@
         <v>300</v>
       </c>
       <c r="I11" s="1">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>40</v>
@@ -4762,7 +4847,7 @@
         <v>41</v>
       </c>
       <c r="M11" s="2">
-        <v>45502.0</v>
+        <v>45502</v>
       </c>
       <c r="Q11" s="1" t="s">
         <v>42</v>
@@ -4786,10 +4871,10 @@
         <v>47</v>
       </c>
       <c r="AB11" s="1">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="AC11" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="AD11" s="1" t="s">
         <v>271</v>
@@ -4798,13 +4883,13 @@
         <v>48</v>
       </c>
       <c r="AG11" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI11" s="1" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>302</v>
       </c>
@@ -4821,7 +4906,7 @@
         <v>303</v>
       </c>
       <c r="I12" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>40</v>
@@ -4830,7 +4915,7 @@
         <v>41</v>
       </c>
       <c r="M12" s="2">
-        <v>45957.0</v>
+        <v>45957</v>
       </c>
       <c r="Q12" s="1" t="s">
         <v>42</v>
@@ -4854,10 +4939,10 @@
         <v>166</v>
       </c>
       <c r="AB12" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="AC12" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="AD12" s="1" t="s">
         <v>266</v>
@@ -4869,13 +4954,13 @@
         <v>48</v>
       </c>
       <c r="AG12" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI12" s="1" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>306</v>
       </c>
@@ -4892,7 +4977,7 @@
         <v>307</v>
       </c>
       <c r="I13" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>40</v>
@@ -4901,7 +4986,7 @@
         <v>41</v>
       </c>
       <c r="M13" s="2">
-        <v>45957.0</v>
+        <v>45957</v>
       </c>
       <c r="Q13" s="1" t="s">
         <v>42</v>
@@ -4925,10 +5010,10 @@
         <v>166</v>
       </c>
       <c r="AB13" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="AC13" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="AD13" s="1" t="s">
         <v>266</v>
@@ -4940,13 +5025,13 @@
         <v>48</v>
       </c>
       <c r="AG13" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI13" s="1" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>309</v>
       </c>
@@ -4963,7 +5048,7 @@
         <v>310</v>
       </c>
       <c r="I14" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="K14" s="1" t="s">
         <v>40</v>
@@ -4972,7 +5057,7 @@
         <v>41</v>
       </c>
       <c r="M14" s="2">
-        <v>46009.0</v>
+        <v>46009</v>
       </c>
       <c r="Q14" s="1" t="s">
         <v>42</v>
@@ -4996,10 +5081,10 @@
         <v>166</v>
       </c>
       <c r="AB14" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="AC14" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="AD14" s="1" t="s">
         <v>266</v>
@@ -5011,13 +5096,13 @@
         <v>48</v>
       </c>
       <c r="AG14" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI14" s="1" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>312</v>
       </c>
@@ -5034,7 +5119,7 @@
         <v>313</v>
       </c>
       <c r="I15" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>40</v>
@@ -5043,7 +5128,7 @@
         <v>41</v>
       </c>
       <c r="M15" s="2">
-        <v>46006.0</v>
+        <v>46006</v>
       </c>
       <c r="Q15" s="1" t="s">
         <v>42</v>
@@ -5067,10 +5152,10 @@
         <v>314</v>
       </c>
       <c r="AB15" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="AC15" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="AD15" s="1" t="s">
         <v>271</v>
@@ -5079,13 +5164,13 @@
         <v>48</v>
       </c>
       <c r="AG15" s="2">
-        <v>45677.0</v>
+        <v>45677</v>
       </c>
       <c r="AI15" s="1" t="s">
         <v>315</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Feat: Forecast commit message
</commit_message>
<xml_diff>
--- a/data/raw/ethiopia_fi_unified_data.xlsx
+++ b/data/raw/ethiopia_fi_unified_data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="5000" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="5000"/>
   </bookViews>
   <sheets>
     <sheet name="ethiopia_fi_unified_data" sheetId="1" r:id="rId1"/>
@@ -3486,6 +3486,9 @@
       <c r="F35" s="1" t="s">
         <v>205</v>
       </c>
+      <c r="H35" s="1">
+        <v>0</v>
+      </c>
       <c r="I35" s="1" t="s">
         <v>206</v>
       </c>
@@ -3542,6 +3545,9 @@
       <c r="F36" s="1" t="s">
         <v>213</v>
       </c>
+      <c r="H36" s="1">
+        <v>0</v>
+      </c>
       <c r="I36" s="1" t="s">
         <v>206</v>
       </c>
@@ -3595,6 +3601,9 @@
       <c r="F37" s="1" t="s">
         <v>219</v>
       </c>
+      <c r="H37" s="1">
+        <v>0</v>
+      </c>
       <c r="I37" s="1" t="s">
         <v>206</v>
       </c>
@@ -3648,6 +3657,9 @@
       <c r="F38" s="1" t="s">
         <v>225</v>
       </c>
+      <c r="H38" s="1">
+        <v>0</v>
+      </c>
       <c r="I38" s="1" t="s">
         <v>206</v>
       </c>
@@ -3704,6 +3716,9 @@
       <c r="F39" s="1" t="s">
         <v>230</v>
       </c>
+      <c r="H39" s="1">
+        <v>0</v>
+      </c>
       <c r="I39" s="1" t="s">
         <v>231</v>
       </c>
@@ -3757,6 +3772,9 @@
       <c r="F40" s="1" t="s">
         <v>236</v>
       </c>
+      <c r="H40" s="1">
+        <v>0</v>
+      </c>
       <c r="I40" s="1" t="s">
         <v>237</v>
       </c>
@@ -3813,6 +3831,9 @@
       <c r="F41" s="1" t="s">
         <v>243</v>
       </c>
+      <c r="H41" s="1">
+        <v>0</v>
+      </c>
       <c r="I41" s="1" t="s">
         <v>206</v>
       </c>
@@ -3866,6 +3887,9 @@
       <c r="F42" s="1" t="s">
         <v>248</v>
       </c>
+      <c r="H42" s="1">
+        <v>0</v>
+      </c>
       <c r="I42" s="1" t="s">
         <v>206</v>
       </c>
@@ -3919,6 +3943,9 @@
       <c r="F43" s="1" t="s">
         <v>253</v>
       </c>
+      <c r="H43" s="1">
+        <v>0</v>
+      </c>
       <c r="I43" s="1" t="s">
         <v>206</v>
       </c>
@@ -3980,6 +4007,9 @@
       </c>
       <c r="F44" s="1" t="s">
         <v>258</v>
+      </c>
+      <c r="H44" s="1">
+        <v>0</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>231</v>

</xml_diff>